<commit_message>
Dashboard: rombak desain grafik + anti-error dengan IFERROR
PERBAIKAN:
- Formula % Surplus Total pakai IFERROR (tidak ada #VALUE! / #DIV/0!)
- Helper data rows 58-63 dengan label pendek: Terpakai/Sisa/Surplus/Defisit
  Semua value di-wrap IFERROR dan MAX(0,...) / ABS() supaya konsisten positif

DESAIN CHART BARU (lebih profesional):
1. Donut 'Penyerapan Anggaran'
   * Label di luar slice (outEnd) dengan separator ': '
   * Border putih 2px tebal antar slice
   * Title UPPERCASE bold biru navy
   * Legend bold di bawah
   * Hole size 60% (lebih lega)

2. Column Chart 'Akumulasi Surplus vs Defisit'
   * Bar vertikal (bukan horizontal) - lebih mudah dibaca
   * Warna solid tanpa border: hijau (surplus) + merah (defisit)
   * Y-axis disembunyikan, gridlines dihilangkan (clean)
   * Label Rp di atas bar (outEnd), font 11pt bold
   * X-axis dengan label bold 12pt
   * Gap width 80% (bar lebih tebal)

LAYOUT:
- Border chart abu-abu 1pt
- Background putih clean
- Font Calibri consistent
</commit_message>
<xml_diff>
--- a/Akumulasi_Total_Enhanced.xlsx
+++ b/Akumulasi_Total_Enhanced.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="151">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="193" uniqueCount="156">
   <si>
     <t>DASHBOARD LAPORAN KEUANGAN</t>
   </si>
@@ -475,6 +475,21 @@
   </si>
   <si>
     <t>% Surplus Total (dari Total Pagu)</t>
+  </si>
+  <si>
+    <t>E. VISUALISASI</t>
+  </si>
+  <si>
+    <t>Terpakai</t>
+  </si>
+  <si>
+    <t>Sisa</t>
+  </si>
+  <si>
+    <t>Surplus</t>
+  </si>
+  <si>
+    <t>Defisit</t>
   </si>
 </sst>
 </file>
@@ -2032,7 +2047,7 @@
           <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" wrap="square" anchor="ctr" anchorCtr="1"/>
           <a:lstStyle/>
           <a:p>
-            <a:pPr>
+            <a:pPr algn="ctr">
               <a:defRPr/>
             </a:pPr>
             <a:r>
@@ -2040,8 +2055,9 @@
                 <a:solidFill>
                   <a:srgbClr val="1F4E79"/>
                 </a:solidFill>
+                <a:latin typeface="Calibri"/>
               </a:rPr>
-              <a:t>Penyerapan Anggaran</a:t>
+              <a:t>PENYERAPAN ANGGARAN</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -2066,7 +2082,7 @@
               <a:solidFill>
                 <a:srgbClr val="ED7D31"/>
               </a:solidFill>
-              <a:ln w="19050">
+              <a:ln w="25400">
                 <a:solidFill>
                   <a:srgbClr val="FFFFFF"/>
                 </a:solidFill>
@@ -2080,7 +2096,7 @@
               <a:solidFill>
                 <a:srgbClr val="70AD47"/>
               </a:solidFill>
-              <a:ln w="19050">
+              <a:ln w="25400">
                 <a:solidFill>
                   <a:srgbClr val="FFFFFF"/>
                 </a:solidFill>
@@ -2092,9 +2108,9 @@
               <a:solidFill>
                 <a:srgbClr val="FFFFFF"/>
               </a:solidFill>
-              <a:ln>
+              <a:ln w="9525">
                 <a:solidFill>
-                  <a:srgbClr val="BFBFBF"/>
+                  <a:srgbClr val="D9D9D9"/>
                 </a:solidFill>
               </a:ln>
             </c:spPr>
@@ -2103,23 +2119,27 @@
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
-                  <a:defRPr sz="1200" b="1"/>
+                  <a:defRPr sz="1100" b="1">
+                    <a:solidFill>
+                      <a:srgbClr val="262626"/>
+                    </a:solidFill>
+                  </a:defRPr>
                 </a:pPr>
                 <a:endParaRPr lang="id-ID"/>
               </a:p>
             </c:txPr>
+            <c:dLblPos val="outEnd"/>
             <c:showLegendKey val="0"/>
             <c:showVal val="0"/>
             <c:showCatName val="1"/>
             <c:showSerName val="0"/>
             <c:showPercent val="1"/>
             <c:showBubbleSize val="0"/>
-            <c:separator>
-</c:separator>
+            <c:separator>: </c:separator>
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>Dashboard!$A$30:$A$31</c:f>
+              <c:f>Dashboard!$A$58:$A$59</c:f>
               <c:strCache>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
@@ -2133,12 +2153,22 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Dashboard!$B$30:$B$31</c:f>
+              <c:f>Dashboard!$B$58:$B$59</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="2"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
             </c:numRef>
           </c:val>
         </c:ser>
         <c:firstSliceAng val="0"/>
-        <c:holeSize val="55"/>
+        <c:holeSize val="60"/>
       </c:doughnutChart>
     </c:plotArea>
     <c:legend>
@@ -2149,7 +2179,7 @@
         <a:lstStyle/>
         <a:p>
           <a:pPr>
-            <a:defRPr sz="1100"/>
+            <a:defRPr sz="1100" b="1"/>
           </a:pPr>
           <a:endParaRPr lang="id-ID"/>
         </a:p>
@@ -2162,9 +2192,9 @@
     <a:solidFill>
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln w="9525">
+    <a:ln w="12700">
       <a:solidFill>
-        <a:srgbClr val="D9D9D9"/>
+        <a:srgbClr val="BFBFBF"/>
       </a:solidFill>
     </a:ln>
   </c:spPr>
@@ -2178,16 +2208,20 @@
     <c:title>
       <c:tx>
         <c:rich>
-          <a:bodyPr/>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" wrap="square" anchor="ctr" anchorCtr="1"/>
           <a:lstStyle/>
           <a:p>
+            <a:pPr algn="ctr">
+              <a:defRPr/>
+            </a:pPr>
             <a:r>
               <a:rPr lang="id-ID" b="1" sz="1400">
                 <a:solidFill>
                   <a:srgbClr val="1F4E79"/>
                 </a:solidFill>
+                <a:latin typeface="Calibri"/>
               </a:rPr>
-              <a:t>Akumulasi Surplus vs Defisit</a:t>
+              <a:t>AKUMULASI SURPLUS vs DEFISIT</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -2198,7 +2232,7 @@
     <c:plotArea>
       <c:layout/>
       <c:barChart>
-        <c:barDir val="bar"/>
+        <c:barDir val="col"/>
         <c:grouping val="clustered"/>
         <c:varyColors val="1"/>
         <c:ser>
@@ -2211,8 +2245,11 @@
             <a:solidFill>
               <a:srgbClr val="70AD47"/>
             </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
           </c:spPr>
-          <c:invertIfNegative val="1"/>
+          <c:invertIfNegative val="0"/>
           <c:dPt>
             <c:idx val="0"/>
             <c:invertIfNegative val="0"/>
@@ -2221,6 +2258,9 @@
               <a:solidFill>
                 <a:srgbClr val="70AD47"/>
               </a:solidFill>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
             </c:spPr>
           </c:dPt>
           <c:dPt>
@@ -2231,6 +2271,9 @@
               <a:solidFill>
                 <a:srgbClr val="C00000"/>
               </a:solidFill>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
             </c:spPr>
           </c:dPt>
           <c:dLbls>
@@ -2239,7 +2282,11 @@
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
-                  <a:defRPr sz="1000" b="1"/>
+                  <a:defRPr sz="1100" b="1">
+                    <a:solidFill>
+                      <a:srgbClr val="262626"/>
+                    </a:solidFill>
+                  </a:defRPr>
                 </a:pPr>
                 <a:endParaRPr lang="id-ID"/>
               </a:p>
@@ -2255,25 +2302,35 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>Dashboard!$A$44:$A$45</c:f>
+              <c:f>Dashboard!$A$62:$A$63</c:f>
               <c:strCache>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>Total Surplus</c:v>
+                  <c:v>Surplus</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>Total Defisit</c:v>
+                  <c:v>Defisit</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Dashboard!$B$44:$B$45</c:f>
+              <c:f>Dashboard!$B$62:$B$63</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="2"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
             </c:numRef>
           </c:val>
         </c:ser>
-        <c:gapWidth val="100"/>
+        <c:gapWidth val="80"/>
         <c:axId val="901"/>
         <c:axId val="902"/>
       </c:barChart>
@@ -2283,16 +2340,28 @@
           <c:orientation val="minMax"/>
         </c:scaling>
         <c:delete val="0"/>
-        <c:axPos val="l"/>
-        <c:majorTickMark val="out"/>
+        <c:axPos val="b"/>
+        <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:solidFill>
+              <a:srgbClr val="BFBFBF"/>
+            </a:solidFill>
+          </a:ln>
+        </c:spPr>
         <c:txPr>
           <a:bodyPr/>
           <a:lstStyle/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="1100" b="1"/>
+              <a:defRPr sz="1200" b="1">
+                <a:solidFill>
+                  <a:srgbClr val="262626"/>
+                </a:solidFill>
+              </a:defRPr>
             </a:pPr>
             <a:endParaRPr lang="id-ID"/>
           </a:p>
@@ -2304,20 +2373,11 @@
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
-        <c:delete val="0"/>
-        <c:axPos val="b"/>
-        <c:majorGridlines>
-          <c:spPr>
-            <a:ln w="9525">
-              <a:solidFill>
-                <a:srgbClr val="E7E6E6"/>
-              </a:solidFill>
-            </a:ln>
-          </c:spPr>
-        </c:majorGridlines>
+        <c:delete val="1"/>
+        <c:axPos val="l"/>
         <c:numFmt formatCode="&quot;Rp&quot;#,##0" sourceLinked="0"/>
-        <c:majorTickMark val="out"/>
-        <c:tickLblPos val="nextTo"/>
+        <c:majorTickMark val="none"/>
+        <c:tickLblPos val="none"/>
         <c:crossAx val="901"/>
       </c:valAx>
       <c:spPr>
@@ -2334,9 +2394,9 @@
     <a:solidFill>
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln w="9525">
+    <a:ln w="12700">
       <a:solidFill>
-        <a:srgbClr val="D9D9D9"/>
+        <a:srgbClr val="BFBFBF"/>
       </a:solidFill>
     </a:ln>
   </c:spPr>
@@ -3100,12 +3160,12 @@
         <v>-6666931</v>
       </c>
     </row>
-    <row r="47" ht="20.25" customHeight="1">
+    <row r="47" ht="22" customHeight="1">
       <c r="A47" s="3" t="s">
         <v>150</v>
       </c>
       <c r="B47" s="21">
-        <f>IF(SUM('Rekap Harian'!$K$6:$K$36)=0,0,B46/SUM('Rekap Harian'!$K$6:$K$36))</f>
+        <f>IFERROR(B46/SUM('Rekap Harian'!$K$6:$K$36),0)</f>
       </c>
     </row>
     <row r="48" ht="15.75" customHeight="1">
@@ -3153,13 +3213,45 @@
       </c>
     </row>
     <row r="56" ht="15.75" customHeight="1"/>
-    <row r="57" ht="15.75" customHeight="1"/>
-    <row r="58" ht="15.75" customHeight="1"/>
-    <row r="59" ht="15.75" customHeight="1"/>
+    <row r="57" ht="20" customHeight="1">
+      <c r="A57" s="17" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="58" ht="18" customHeight="1">
+      <c r="A58" s="10" t="s">
+        <v>152</v>
+      </c>
+      <c r="B58" s="24">
+        <f>IFERROR(B30,0)</f>
+      </c>
+    </row>
+    <row r="59" ht="18" customHeight="1">
+      <c r="A59" s="10" t="s">
+        <v>153</v>
+      </c>
+      <c r="B59" s="24">
+        <f>IFERROR(MAX(0,B31),0)</f>
+      </c>
+    </row>
+    <row r="62" ht="18" customHeight="1">
+      <c r="A62" s="10" t="s">
+        <v>154</v>
+      </c>
+      <c r="B62" s="24">
+        <f>IFERROR(B44,0)</f>
+      </c>
+    </row>
+    <row r="63" ht="18" customHeight="1">
+      <c r="A63" s="10" t="s">
+        <v>155</v>
+      </c>
+      <c r="B63" s="24">
+        <f>IFERROR(ABS(B45),0)</f>
+      </c>
+    </row>
     <row r="60" ht="15.75" customHeight="1"/>
     <row r="61" ht="15.75" customHeight="1"/>
-    <row r="62" ht="15.75" customHeight="1"/>
-    <row r="63" ht="15.75" customHeight="1"/>
     <row r="64" ht="15.75" customHeight="1"/>
     <row r="65" ht="15.75" customHeight="1"/>
     <row r="66" ht="15.75" customHeight="1"/>

</xml_diff>